<commit_message>
Sincronización automática de DETALLE_PERSONAL_OBRAS.xlsx
</commit_message>
<xml_diff>
--- a/DETALLE_PERSONAL_OBRAS.xlsx
+++ b/DETALLE_PERSONAL_OBRAS.xlsx
@@ -508,15 +508,6 @@
           <t>00-OFICINA</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#00-OFICINA/00-OFICINA_KML.kml</t>
@@ -555,15 +546,6 @@
           <t>AGS COSTA DEL SOL HAZA DEL CONDE</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AGS COSTA DEL SOL HAZA DEL CONDE/AGS COSTA DEL SOL HAZA DEL CONDE_KML.kml</t>
@@ -604,15 +586,6 @@
           <t>AMCONSTRUCCIONES BENAHAVIS</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AMCONSTRUCCIONES BENAHAVIS/AMCONSTRUCCIONES BENAHAVIS_KML.kml</t>
@@ -667,15 +640,6 @@
           <t>ARTE2 CALLE ALBERTI</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#ARTE2 CALLE ALBERTI/ARTE2 CALLE ALBERTI_KML.kml</t>
@@ -738,15 +702,6 @@
           <t>ARTE2 SAN PEDRO</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#ARTE2 SAN PEDRO/ARTE2 SAN PEDRO_KML.kml</t>
@@ -789,15 +744,6 @@
           <t>AVENTUS BENALMADENA</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AVENTUS BENALMADENA/AVENTUS BENALMADENA_KML.kml</t>
@@ -840,15 +786,6 @@
           <t>AVENTUS EL ROSARIO</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AVENTUS EL ROSARIO/AVENTUS EL ROSARIO_KML.kml</t>
@@ -897,15 +834,6 @@
           <t>AVENTUS ELALMENDRO</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AVENTUS ELALMENDRO/AVENTUS ELALMENDRO_KML.kml</t>
@@ -990,15 +918,6 @@
           <t>AVENTUS MARBESA</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AVENTUS MARBESA/AVENTUS MARBESA_KML.kml</t>
@@ -1083,15 +1002,6 @@
           <t>AVENTUS NAGUELES</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AVENTUS NAGUELES/AVENTUS NAGUELES_KML.kml</t>
@@ -1134,15 +1044,6 @@
           <t>AVENTUS PUENTE ROMANO</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AVENTUS PUENTE ROMANO/AVENTUS PUENTE ROMANO_KML.kml</t>
@@ -1183,15 +1084,6 @@
           <t>Aventus Puente Romano 123</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#Aventus Puente Romano 123/Aventus Puente Romano 123_KML.kml</t>
@@ -1232,15 +1124,6 @@
           <t>AYELEN LA VINUELA F2</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AYELEN LA VINUELA F2/AYELEN LA VINUELA F2_KML.kml</t>
@@ -1317,15 +1200,6 @@
           <t>AYELEN LA VINUELA F3</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#AYELEN LA VINUELA F3/AYELEN LA VINUELA F3_KML.kml</t>
@@ -1372,15 +1246,6 @@
           <t>BILBA 32 VIV MIJAS</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA 32 VIV MIJAS/BILBA 32 VIV MIJAS_KML.kml</t>
@@ -1429,15 +1294,6 @@
           <t>BILBA 50 VIV SAN LUCAS</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA 50 VIV SAN LUCAS/BILBA 50 VIV SAN LUCAS_KML.kml</t>
@@ -1520,15 +1376,6 @@
           <t>BILBA 67 VIV CARTAMA</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA 67 VIV CARTAMA/BILBA 67 VIV CARTAMA_KML.kml</t>
@@ -1603,15 +1450,6 @@
           <t>BILBA CALLE ALMOTAJE</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA CALLE ALMOTAJE/BILBA CALLE ALMOTAJE_KML.kml</t>
@@ -1662,15 +1500,6 @@
           <t>BILBA CORTIJO_MERINO</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA CORTIJO_MERINO/BILBA CORTIJO_MERINO_KML.kml</t>
@@ -2109,15 +1938,6 @@
           <t>BILBA DISTRITOZETA</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA DISTRITOZETA/BILBA DISTRITOZETA_KML.kml</t>
@@ -2180,15 +2000,6 @@
           <t>BILBA HOSPITAL MATERNO INFANTIL</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA HOSPITAL MATERNO INFANTIL/BILBA HOSPITAL MATERNO INFANTIL_KML.kml</t>
@@ -2251,15 +2062,6 @@
           <t>BILBA MAIA</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA MAIA/BILBA MAIA_KML.kml</t>
@@ -2296,15 +2098,6 @@
           <t>BILBA SANTA MARIA GOLF</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#BILBA SANTA MARIA GOLF/BILBA SANTA MARIA GOLF_KML.kml</t>
@@ -2345,15 +2138,6 @@
           <t>CALDERON BAY8-BAY7</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CALDERON BAY8-BAY7/CALDERON BAY8-BAY7_KML.kml</t>
@@ -2482,15 +2266,6 @@
           <t>CALDERON SANTA ELENA</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CALDERON SANTA ELENA/CALDERON SANTA ELENA_KML.kml</t>
@@ -2533,15 +2308,6 @@
           <t>CAMINO BENAHAVIS</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CAMINO BENAHAVIS/CAMINO BENAHAVIS_KML.kml</t>
@@ -2718,15 +2484,6 @@
           <t>CARPESOL CHAPARRAL</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CARPESOL CHAPARRAL/CARPESOL CHAPARRAL_KML.kml</t>
@@ -2807,15 +2564,6 @@
           <t>CARPESOL LA CALA</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CARPESOL LA CALA/CARPESOL LA CALA_KML.kml</t>
@@ -2868,15 +2616,6 @@
           <t>CARPESOL MACAN</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CARPESOL MACAN/CARPESOL MACAN_KML.kml</t>
@@ -3073,15 +2812,6 @@
           <t>Chamorro Alhaurin</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#Chamorro Alhaurin/Chamorro Alhaurin_KML.kml</t>
@@ -3128,15 +2858,6 @@
           <t>CHIRIVO 120 VIV ALTO DEL CHAPARRAL</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CHIRIVO 120 VIV ALTO DEL CHAPARRAL/CHIRIVO 120 VIV ALTO DEL CHAPARRAL_KML.kml</t>
@@ -3303,15 +3024,6 @@
           <t>CHIRIVO 46 VIV EL CHAPARRAL</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CHIRIVO 46 VIV EL CHAPARRAL/CHIRIVO 46 VIV EL CHAPARRAL_KML.kml</t>
@@ -3544,15 +3256,6 @@
           <t>CHIRIVO 48 VIV EL ROMERAL</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CHIRIVO 48 VIV EL ROMERAL/CHIRIVO 48 VIV EL ROMERAL_KML.kml</t>
@@ -3593,15 +3296,6 @@
           <t>CHIRIVO OLIVARA LIVING</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CHIRIVO OLIVARA LIVING/CHIRIVO OLIVARA LIVING_KML.kml</t>
@@ -3640,15 +3334,6 @@
           <t>CHIRIVO PROMAR 20 Y 31 VIV</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CHIRIVO PROMAR 20 Y 31 VIV/CHIRIVO PROMAR 20 Y 31 VIV_KML.kml</t>
@@ -3715,15 +3400,6 @@
           <t>CONSTRUMARBEL ALHAMVRA</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CONSTRUMARBEL ALHAMVRA/CONSTRUMARBEL ALHAMVRA_KML.kml</t>
@@ -3762,15 +3438,6 @@
           <t>CONSTRUMARBEL SIBELIUS</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CONSTRUMARBEL SIBELIUS/CONSTRUMARBEL SIBELIUS_KML.kml</t>
@@ -3829,15 +3496,6 @@
           <t>CONSTRUMARBEL SOTOGRANDE</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CONSTRUMARBEL SOTOGRANDE/CONSTRUMARBEL SOTOGRANDE_KML.kml</t>
@@ -3892,15 +3550,6 @@
           <t>CORAL SANTANGELO 139</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#CORAL SANTANGELO 139/CORAL SANTANGELO 139_KML.kml</t>
@@ -3971,15 +3620,6 @@
           <t>COSENTRANS CONDE DE URENA</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#COSENTRANS CONDE DE URENA/COSENTRANS CONDE DE URENA_KML.kml</t>
@@ -4022,15 +3662,6 @@
           <t>DESARROLLA ESTEPONA</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#DESARROLLA ESTEPONA/DESARROLLA ESTEPONA_KML.kml</t>
@@ -4199,15 +3830,6 @@
           <t>DOMUS CODORNIZ155</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#DOMUS CODORNIZ155/DOMUS CODORNIZ155_KML.kml</t>
@@ -4264,15 +3886,6 @@
           <t>EGT CALLE_REAL</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#EGT CALLE_REAL/EGT CALLE_REAL_KML.kml</t>
@@ -4325,15 +3938,6 @@
           <t>EGT TORREMOLINOS</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#EGT TORREMOLINOS/EGT TORREMOLINOS_KML.kml</t>
@@ -4394,15 +3998,6 @@
           <t>EMILE G2</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#EMILE G2/EMILE G2_KML.kml</t>
@@ -4445,15 +4040,6 @@
           <t>EMILE LA QUINTA</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#EMILE LA QUINTA/EMILE LA QUINTA_KML.kml</t>
@@ -4496,15 +4082,6 @@
           <t>EMILE ZAGALETA</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#EMILE ZAGALETA/EMILE ZAGALETA_KML.kml</t>
@@ -4559,15 +4136,6 @@
           <t>ESPIREA HIPODROMO</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#ESPIREA HIPODROMO/ESPIREA HIPODROMO_KML.kml</t>
@@ -4620,15 +4188,6 @@
           <t>ESPIREA NAVIGOLF</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#ESPIREA NAVIGOLF/ESPIREA NAVIGOLF_KML.kml</t>
@@ -4713,15 +4272,6 @@
           <t>FECADA CERRADO DEL AGILA</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#FECADA CERRADO DEL AGILA/FECADA CERRADO DEL AGILA_KML.kml</t>
@@ -4760,15 +4310,6 @@
           <t>FECADA LOS PACOS</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#FECADA LOS PACOS/FECADA LOS PACOS_KML.kml</t>
@@ -4811,15 +4352,6 @@
           <t>FMG SANTANGELO</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#FMG SANTANGELO/FMG SANTANGELO_KML.kml</t>
@@ -4862,15 +4394,6 @@
           <t>FONSAN CARTAMA</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#FONSAN CARTAMA/FONSAN CARTAMA_KML.kml</t>
@@ -4963,15 +4486,6 @@
           <t>FRAM LANTANA</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#FRAM LANTANA/FRAM LANTANA_KML.kml</t>
@@ -5072,15 +4586,6 @@
           <t>FRAM SOTOGRANDE</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#FRAM SOTOGRANDE/FRAM SOTOGRANDE_KML.kml</t>
@@ -5119,15 +4624,6 @@
           <t>GAILUR BENALUS</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#GAILUR BENALUS/GAILUR BENALUS_KML.kml</t>
@@ -5258,15 +4754,6 @@
           <t>GARCU MANILVA</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#GARCU MANILVA/GARCU MANILVA_KML.kml</t>
@@ -5307,15 +4794,6 @@
           <t>GEORREFERENCIAR</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#GEORREFERENCIAR/GEORREFERENCIAR_KML.kml</t>
@@ -5358,15 +4836,6 @@
           <t>GOMEZTRANS SANTANGELO</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#GOMEZTRANS SANTANGELO/GOMEZTRANS SANTANGELO_KML.kml</t>
@@ -5415,15 +4884,6 @@
           <t>GRUPOPISCIS TERMICA</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#GRUPOPISCIS TERMICA/GRUPOPISCIS TERMICA_KML.kml</t>
@@ -5646,15 +5106,6 @@
           <t>HERYSAN ELYSIA</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#HERYSAN ELYSIA/HERYSAN ELYSIA_KML.kml</t>
@@ -5693,15 +5144,6 @@
           <t>IELCO 66 VIV MEZQUITILLA</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#IELCO 66 VIV MEZQUITILLA/IELCO 66 VIV MEZQUITILLA_KML.kml</t>
@@ -5768,15 +5210,6 @@
           <t>INMOLUX EL MADRO¥AL</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#INMOLUX EL MADRO¥AL/INMOLUX EL MADRO¥AL_KML.kml</t>
@@ -5853,15 +5286,6 @@
           <t>INMOPORSAN 73 VIV ALHAURIN</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#INMOPORSAN 73 VIV ALHAURIN/INMOPORSAN 73 VIV ALHAURIN_KML.kml</t>
@@ -5910,15 +5334,6 @@
           <t>INMOPORSAN ALOZAINA</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#INMOPORSAN ALOZAINA/INMOPORSAN ALOZAINA_KML.kml</t>
@@ -5963,15 +5378,6 @@
           <t>INMOPORSAN CANAVERAL</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#INMOPORSAN CANAVERAL/INMOPORSAN CANAVERAL_KML.kml</t>
@@ -6014,15 +5420,6 @@
           <t>IVAN SANCHEZ PALACIO CONGRESOS</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#IVAN SANCHEZ PALACIO CONGRESOS/IVAN SANCHEZ PALACIO CONGRESOS_KML.kml</t>
@@ -6063,15 +5460,6 @@
           <t>JARALIA SANROQUE</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#JARALIA SANROQUE/JARALIA SANROQUE_KML.kml</t>
@@ -6130,15 +5518,6 @@
           <t>JESUS ESTEPA CALLE ESCORIAL</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#JESUS ESTEPA CALLE ESCORIAL/JESUS ESTEPA CALLE ESCORIAL_KML.kml</t>
@@ -6183,15 +5562,6 @@
           <t>JESUS ESTEPA CALLE OSLO</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#JESUS ESTEPA CALLE OSLO/JESUS ESTEPA CALLE OSLO_KML.kml</t>
@@ -6230,15 +5600,6 @@
           <t>JNG TORROX</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#JNG TORROX/JNG TORROX_KML.kml</t>
@@ -6283,15 +5644,6 @@
           <t>LACOSTA ALHAURIN</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#LACOSTA ALHAURIN/LACOSTA ALHAURIN_KML.kml</t>
@@ -6350,15 +5702,6 @@
           <t>LACOSTA CALAHONDA</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#LACOSTA CALAHONDA/LACOSTA CALAHONDA_KML.kml</t>
@@ -6501,15 +5844,6 @@
           <t>LACOSTA CALLE HOTENSIA</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#LACOSTA CALLE HOTENSIA/LACOSTA CALLE HOTENSIA_KML.kml</t>
@@ -6548,15 +5882,6 @@
           <t>LEBA C GAUCIN</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#LEBA C GAUCIN/LEBA C GAUCIN_KML.kml</t>
@@ -6609,15 +5934,6 @@
           <t>LEBA CABOPINO</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#LEBA CABOPINO/LEBA CABOPINO_KML.kml</t>
@@ -6724,15 +6040,6 @@
           <t>Leba Calle Balcon</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#Leba Calle Balcon/Leba Calle Balcon_KML.kml</t>
@@ -6783,15 +6090,6 @@
           <t>LEBA CALLEANCHA</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#LEBA CALLEANCHA/LEBA CALLEANCHA_KML.kml</t>
@@ -6838,15 +6136,6 @@
           <t>LEBA MARBESA</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#LEBA MARBESA/LEBA MARBESA_KML.kml</t>
@@ -6887,15 +6176,6 @@
           <t>MIGUEL CALLE TIMON</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#MIGUEL CALLE TIMON/MIGUEL CALLE TIMON_KML.kml</t>
@@ -6934,15 +6214,6 @@
           <t>NICHEOFFICE LA PALOMA</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#NICHEOFFICE LA PALOMA/NICHEOFFICE LA PALOMA_KML.kml</t>
@@ -6987,15 +6258,6 @@
           <t>OSCAR SANCHEZ SIERRAZUELO</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#OSCAR SANCHEZ SIERRAZUELO/OSCAR SANCHEZ SIERRAZUELO_KML.kml</t>
@@ -7040,15 +6302,6 @@
           <t>PATRICIO EL MADRONAL</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#PATRICIO EL MADRONAL/PATRICIO EL MADRONAL_KML.kml</t>
@@ -7089,15 +6342,6 @@
           <t>QUABIT 75 VIV</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#QUABIT 75 VIV/QUABIT 75 VIV_KML.kml</t>
@@ -7144,15 +6388,6 @@
           <t>Quabit Churriana 32 viv</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#Quabit Churriana 32 viv/Quabit Churriana 32 viv_KML.kml</t>
@@ -7201,15 +6436,6 @@
           <t>Quabit Churriana 32 viv Estrella</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#Quabit Churriana 32 viv Estrella/Quabit Churriana 32 viv Estrella_KML.kml</t>
@@ -7248,15 +6474,6 @@
           <t>SALADO ADENDIA</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO ADENDIA/SALADO ADENDIA_KML.kml</t>
@@ -7299,15 +6516,6 @@
           <t>SALADO BENAJAFE 2</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO BENAJAFE 2/SALADO BENAJAFE 2_KML.kml</t>
@@ -7378,15 +6586,6 @@
           <t>SALADO BENAJARAFE</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO BENAJARAFE/SALADO BENAJARAFE_KML.kml</t>
@@ -7437,15 +6636,6 @@
           <t>SALADO CALLE ESLIEGO</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO CALLE ESLIEGO/SALADO CALLE ESLIEGO_KML.kml</t>
@@ -7494,15 +6684,6 @@
           <t>SALADO COLINAS DEL LIMONAR</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO COLINAS DEL LIMONAR/SALADO COLINAS DEL LIMONAR_KML.kml</t>
@@ -7549,15 +6730,6 @@
           <t>SALADO CRUZ HUMILLADEROS</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO CRUZ HUMILLADEROS/SALADO CRUZ HUMILLADEROS_KML.kml</t>
@@ -7598,15 +6770,6 @@
           <t>SALADO LIMONAR</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO LIMONAR/SALADO LIMONAR_KML.kml</t>
@@ -7655,15 +6818,6 @@
           <t>SALADO LOS MILANOS</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO LOS MILANOS/SALADO LOS MILANOS_KML.kml</t>
@@ -7702,15 +6856,6 @@
           <t>SALADO PINARES SAN ANTON</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO PINARES SAN ANTON/SALADO PINARES SAN ANTON_KML.kml</t>
@@ -7749,15 +6894,6 @@
           <t>SALADO ROGELIO_OLIVA</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SALADO ROGELIO_OLIVA/SALADO ROGELIO_OLIVA_KML.kml</t>
@@ -7800,15 +6936,6 @@
           <t>SEXMO CARTAMA</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#SEXMO CARTAMA/SEXMO CARTAMA_KML.kml</t>
@@ -7847,15 +6974,6 @@
           <t>UKO</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#UKO/UKO_KML.kml</t>
@@ -7916,15 +7034,6 @@
           <t>VALDICIO</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#VALDICIO/VALDICIO_KML.kml</t>
@@ -8049,15 +7158,6 @@
           <t>VDR NERJA</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#VDR NERJA/VDR NERJA_KML.kml</t>
@@ -8126,15 +7226,6 @@
           <t>VDR TORREBLANCA</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
-      <c r="D102" t="inlineStr"/>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#VDR TORREBLANCA/VDR TORREBLANCA_KML.kml</t>
@@ -8381,15 +7472,6 @@
           <t>ZOLIAR EL PARAISO</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr"/>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
           <t>https://e.pcloud.link/publink/show?code=kZxO5X7ZzkLiRJzJO35y6cnBUHoTfBSuKP97#ZOLIAR EL PARAISO/ZOLIAR EL PARAISO_KML.kml</t>

</xml_diff>